<commit_message>
lo dejamos andando la parte de importar archivos y falta las tareas de ya
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ale\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ale\Documents\GitHub\appPuntoVenta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF611CD-145E-4F5D-844D-9E8030606A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEA8858-A15D-4480-BCDE-06863D54B44F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{77ACDAD0-E555-4A29-BD8E-0943A0472C95}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
   <si>
     <t>agua</t>
   </si>
@@ -97,6 +97,12 @@
   </si>
   <si>
     <t>categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcohol etilico 250 ml  </t>
+  </si>
+  <si>
+    <t>limpieza</t>
   </si>
 </sst>
 </file>
@@ -132,8 +138,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,11 +455,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55D29BEC-D929-4E5B-9298-3BBD69B61605}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" customWidth="1"/>
     <col min="5" max="5" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -725,6 +732,23 @@
         <v>7</v>
       </c>
     </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1">
+        <v>7790139000462</v>
+      </c>
+      <c r="C17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17">
+        <v>2000</v>
+      </c>
+      <c r="E17" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>